<commit_message>
Daily slate 2026-06-25 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-23.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-23.xlsx
@@ -503,13 +503,13 @@
         <v>17</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>64.7</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>326</v>
+        <v>351</v>
       </c>
       <c r="E4" t="n">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="F4" t="n">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="G4" t="n">
-        <v>44.5</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>251</v>
+        <v>276</v>
       </c>
       <c r="E7" t="n">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="F7" t="n">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="G7" t="n">
-        <v>48.2</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -645,13 +645,13 @@
         <v>262</v>
       </c>
       <c r="E8" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F8" t="n">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G8" t="n">
-        <v>22.1</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="9">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G9" t="n">
-        <v>53.1</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="10">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E10" t="n">
         <v>96</v>
       </c>
       <c r="F10" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G10" t="n">
-        <v>50.3</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1186</v>
+        <v>1328</v>
       </c>
       <c r="E11" t="n">
-        <v>736</v>
+        <v>799</v>
       </c>
       <c r="F11" t="n">
-        <v>450</v>
+        <v>529</v>
       </c>
       <c r="G11" t="n">
-        <v>62.1</v>
+        <v>60.2</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="E12" t="n">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="F12" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="G12" t="n">
-        <v>70.59999999999999</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13">
@@ -790,13 +790,13 @@
         <v>292</v>
       </c>
       <c r="E13" t="n">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="F13" t="n">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="G13" t="n">
-        <v>40.1</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="14">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>327</v>
+        <v>357</v>
       </c>
       <c r="E14" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F14" t="n">
-        <v>249</v>
+        <v>277</v>
       </c>
       <c r="G14" t="n">
-        <v>23.9</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>449</v>
+        <v>485</v>
       </c>
       <c r="E15" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F15" t="n">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="G15" t="n">
-        <v>20</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="16">
@@ -874,16 +874,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="E16" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F16" t="n">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="G16" t="n">
-        <v>22.8</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="17">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5747</v>
+        <v>6256</v>
       </c>
       <c r="E17" t="n">
-        <v>1139</v>
+        <v>1190</v>
       </c>
       <c r="F17" t="n">
-        <v>4608</v>
+        <v>5066</v>
       </c>
       <c r="G17" t="n">
-        <v>19.8</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1444,52 +1444,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50.3</v>
+        <v>50</v>
       </c>
       <c r="C7" t="n">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D7" t="n">
-        <v>62.1</v>
+        <v>60.2</v>
       </c>
       <c r="E7" t="n">
-        <v>1186</v>
+        <v>1328</v>
       </c>
       <c r="F7" t="n">
-        <v>70.59999999999999</v>
+        <v>69</v>
       </c>
       <c r="G7" t="n">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="H7" t="n">
-        <v>40.1</v>
+        <v>35.6</v>
       </c>
       <c r="I7" t="n">
         <v>292</v>
       </c>
       <c r="J7" t="n">
-        <v>23.9</v>
+        <v>22.4</v>
       </c>
       <c r="K7" t="n">
-        <v>327</v>
+        <v>357</v>
       </c>
       <c r="L7" t="n">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="M7" t="n">
-        <v>449</v>
+        <v>485</v>
       </c>
       <c r="N7" t="n">
-        <v>22.8</v>
+        <v>21.6</v>
       </c>
       <c r="O7" t="n">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="P7" t="n">
-        <v>19.8</v>
+        <v>19</v>
       </c>
       <c r="Q7" t="n">
-        <v>5747</v>
+        <v>6256</v>
       </c>
       <c r="R7" t="n">
         <v>70.59999999999999</v>
@@ -1498,22 +1498,22 @@
         <v>34</v>
       </c>
       <c r="T7" t="n">
-        <v>44.5</v>
+        <v>43</v>
       </c>
       <c r="U7" t="n">
-        <v>326</v>
+        <v>351</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>22.1</v>
+        <v>21.4</v>
       </c>
       <c r="Y7" t="n">
         <v>262</v>
       </c>
       <c r="Z7" t="n">
-        <v>64.7</v>
+        <v>76.5</v>
       </c>
       <c r="AA7" t="n">
         <v>17</v>
@@ -1525,16 +1525,16 @@
         <v>2</v>
       </c>
       <c r="AD7" t="n">
-        <v>48.2</v>
+        <v>50</v>
       </c>
       <c r="AE7" t="n">
-        <v>251</v>
+        <v>276</v>
       </c>
       <c r="AF7" t="n">
-        <v>53.1</v>
+        <v>53.8</v>
       </c>
       <c r="AG7" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-06-27 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-23.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-23.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E4" t="n">
         <v>151</v>
       </c>
       <c r="F4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G4" t="n">
-        <v>43</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="5">
@@ -642,16 +642,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>262</v>
+        <v>101</v>
       </c>
       <c r="E8" t="n">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="F8" t="n">
-        <v>206</v>
+        <v>62</v>
       </c>
       <c r="G8" t="n">
-        <v>21.4</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="9">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>192</v>
+        <v>511</v>
       </c>
       <c r="E10" t="n">
-        <v>96</v>
+        <v>212</v>
       </c>
       <c r="F10" t="n">
-        <v>96</v>
+        <v>299</v>
       </c>
       <c r="G10" t="n">
-        <v>50</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="11">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1328</v>
+        <v>1363</v>
       </c>
       <c r="E11" t="n">
-        <v>799</v>
+        <v>808</v>
       </c>
       <c r="F11" t="n">
-        <v>529</v>
+        <v>555</v>
       </c>
       <c r="G11" t="n">
-        <v>60.2</v>
+        <v>59.3</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="E12" t="n">
         <v>138</v>
       </c>
       <c r="F12" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G12" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13">
@@ -787,16 +787,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="E13" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F13" t="n">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="G13" t="n">
-        <v>35.6</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="14">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>357</v>
+        <v>546</v>
       </c>
       <c r="E14" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="F14" t="n">
-        <v>277</v>
+        <v>452</v>
       </c>
       <c r="G14" t="n">
-        <v>22.4</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>485</v>
+        <v>1707</v>
       </c>
       <c r="E15" t="n">
-        <v>96</v>
+        <v>197</v>
       </c>
       <c r="F15" t="n">
-        <v>389</v>
+        <v>1510</v>
       </c>
       <c r="G15" t="n">
-        <v>19.8</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="16">
@@ -874,16 +874,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E16" t="n">
         <v>44</v>
       </c>
       <c r="F16" t="n">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G16" t="n">
-        <v>21.6</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="17">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6256</v>
+        <v>4654</v>
       </c>
       <c r="E17" t="n">
-        <v>1190</v>
+        <v>963</v>
       </c>
       <c r="F17" t="n">
-        <v>5066</v>
+        <v>3691</v>
       </c>
       <c r="G17" t="n">
-        <v>19</v>
+        <v>20.7</v>
       </c>
     </row>
   </sheetData>
@@ -1213,52 +1213,52 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28.7</v>
+        <v>34.6</v>
       </c>
       <c r="C4" t="n">
-        <v>94</v>
+        <v>413</v>
       </c>
       <c r="D4" t="n">
-        <v>47.4</v>
+        <v>36</v>
       </c>
       <c r="E4" t="n">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="F4" t="n">
-        <v>63.6</v>
+        <v>43.8</v>
       </c>
       <c r="G4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H4" t="n">
-        <v>100</v>
+        <v>41.7</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J4" t="n">
-        <v>50</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>4</v>
+        <v>193</v>
       </c>
       <c r="L4" t="n">
-        <v>11.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>9</v>
+        <v>1231</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P4" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="Q4" t="n">
-        <v>1635</v>
+        <v>20</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -1270,10 +1270,10 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>17</v>
+        <v>43.6</v>
       </c>
       <c r="Y4" t="n">
-        <v>200</v>
+        <v>39</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
@@ -1444,52 +1444,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>41.5</v>
       </c>
       <c r="C7" t="n">
-        <v>192</v>
+        <v>511</v>
       </c>
       <c r="D7" t="n">
-        <v>60.2</v>
+        <v>59.3</v>
       </c>
       <c r="E7" t="n">
-        <v>1328</v>
+        <v>1363</v>
       </c>
       <c r="F7" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G7" t="n">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="H7" t="n">
-        <v>35.6</v>
+        <v>35.2</v>
       </c>
       <c r="I7" t="n">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="J7" t="n">
-        <v>22.4</v>
+        <v>17.2</v>
       </c>
       <c r="K7" t="n">
-        <v>357</v>
+        <v>546</v>
       </c>
       <c r="L7" t="n">
-        <v>19.8</v>
+        <v>11.5</v>
       </c>
       <c r="M7" t="n">
-        <v>485</v>
+        <v>1707</v>
       </c>
       <c r="N7" t="n">
-        <v>21.6</v>
+        <v>21.4</v>
       </c>
       <c r="O7" t="n">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="P7" t="n">
-        <v>19</v>
+        <v>20.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>6256</v>
+        <v>4654</v>
       </c>
       <c r="R7" t="n">
         <v>70.59999999999999</v>
@@ -1498,19 +1498,19 @@
         <v>34</v>
       </c>
       <c r="T7" t="n">
-        <v>43</v>
+        <v>42.9</v>
       </c>
       <c r="U7" t="n">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>21.4</v>
+        <v>38.6</v>
       </c>
       <c r="Y7" t="n">
-        <v>262</v>
+        <v>101</v>
       </c>
       <c r="Z7" t="n">
         <v>76.5</v>

</xml_diff>